<commit_message>
Facebook tile system: Style 3 gradient + Style 2 infographic templates + first 5 queue tiles
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/growth-marketing/facebook-content/Facebook Content Calendar.xlsx
+++ b/growth-marketing/facebook-content/Facebook Content Calendar.xlsx
@@ -660,7 +660,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr"/>
@@ -811,7 +811,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr"/>
@@ -864,7 +864,7 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr"/>
@@ -966,7 +966,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr"/>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="K12" s="7" t="inlineStr"/>

</xml_diff>